<commit_message>
Local changes before pulling
</commit_message>
<xml_diff>
--- a/uploads/dlf.xlsx
+++ b/uploads/dlf.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ChandraRealtors\Data\Bhaiya\"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2645" uniqueCount="2593">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2670" uniqueCount="2603">
   <si>
     <t>OWNER'S NAME</t>
   </si>
@@ -7799,6 +7799,39 @@
   </si>
   <si>
     <t>Remark</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t xml:space="preserve">hello
+</t>
+  </si>
+  <si>
+    <t>ranjeet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
+    <t>REMARKS</t>
+  </si>
+  <si>
+    <t>Hiii</t>
+  </si>
+  <si>
+    <t>remark</t>
+  </si>
+  <si>
+    <t>hello</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REMARKS
+</t>
+  </si>
+  <si>
+    <t>dealy</t>
   </si>
 </sst>
 </file>
@@ -8492,18 +8525,18 @@
   <dimension ref="A1:N671"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="38" style="49" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" hidden="1"/>
-    <col min="3" max="3" width="12" hidden="1"/>
-    <col min="4" max="4" width="12.7109375" hidden="1"/>
-    <col min="5" max="5" width="11.140625" hidden="1"/>
-    <col min="6" max="7" width="9.140625" hidden="1"/>
-    <col min="8" max="8" width="21.85546875" hidden="1"/>
-    <col min="9" max="9" width="75.140625" hidden="1"/>
-    <col min="10" max="10" width="20.7109375" style="49" customWidth="1"/>
-    <col min="11" max="11" width="0.42578125" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="18.7109375" hidden="1"/>
-    <col min="13" max="245" width="10" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" style="49" width="38.0"/>
+    <col min="2" max="2" hidden="true" width="9.140625"/>
+    <col min="3" max="3" hidden="true" width="12.0"/>
+    <col min="4" max="4" hidden="true" width="12.7109375"/>
+    <col min="5" max="5" hidden="true" width="11.140625"/>
+    <col min="6" max="7" hidden="true" width="9.140625"/>
+    <col min="8" max="8" hidden="true" width="21.85546875"/>
+    <col min="9" max="9" hidden="true" width="75.140625"/>
+    <col min="10" max="10" customWidth="true" style="49" width="20.7109375"/>
+    <col min="11" max="11" customWidth="true" hidden="true" width="0.42578125"/>
+    <col min="12" max="12" hidden="true" width="18.7109375"/>
+    <col min="13" max="245" customWidth="true" width="10.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="20.25">
@@ -8519,8 +8552,15 @@
       <c r="H1" s="68"/>
       <c r="I1" s="68"/>
       <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
+      <c r="K1" s="68" t="s">
+        <v>2596</v>
+      </c>
+      <c r="L1" s="68" t="s">
+        <v>2596</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>2593</v>
+      </c>
     </row>
     <row r="2" spans="1:14" ht="18.75">
       <c r="A2" s="69" t="s">
@@ -8553,10 +8593,12 @@
       <c r="J2" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="73"/>
+      <c r="K2" s="73" t="s">
+        <v>2599</v>
+      </c>
       <c r="L2" s="70"/>
       <c r="M2" s="74" t="s">
-        <v>2592</v>
+        <v>2599</v>
       </c>
       <c r="N2" s="75"/>
     </row>
@@ -8587,9 +8629,13 @@
       <c r="J3" s="51">
         <v>9958291116</v>
       </c>
-      <c r="K3" s="3"/>
+      <c r="K3" s="3" t="s">
+        <v>2600</v>
+      </c>
       <c r="L3" s="5"/>
-      <c r="M3" s="6"/>
+      <c r="M3" s="6" t="s">
+        <v>2602</v>
+      </c>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="45" t="s">
@@ -8621,6 +8667,9 @@
       <c r="K4" s="3"/>
       <c r="L4" s="2"/>
       <c r="M4" s="6"/>
+      <c r="N4" t="s" s="0">
+        <v>2593</v>
+      </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="45" t="s">
@@ -8649,9 +8698,13 @@
       <c r="J5" s="53">
         <v>9818850260</v>
       </c>
-      <c r="K5" s="3"/>
+      <c r="K5" s="3" t="s">
+        <v>2600</v>
+      </c>
       <c r="L5" s="5"/>
-      <c r="M5" s="6"/>
+      <c r="M5" s="6" t="s">
+        <v>2598</v>
+      </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="45" t="s">
@@ -8710,7 +8763,9 @@
         <v>9811768917</v>
       </c>
       <c r="K7" s="3"/>
-      <c r="L7" s="2"/>
+      <c r="L7" s="2" t="s">
+        <v>2593</v>
+      </c>
       <c r="M7" s="6"/>
     </row>
     <row r="8" spans="1:14">
@@ -8741,7 +8796,9 @@
         <v>9810062994</v>
       </c>
       <c r="K8" s="3"/>
-      <c r="L8" s="2"/>
+      <c r="L8" s="2" t="s">
+        <v>2593</v>
+      </c>
       <c r="M8" s="6"/>
     </row>
     <row r="9" spans="1:14">

</xml_diff>